<commit_message>
7.5: presupuesto de creadores y compromiso congelado
BR-CAMPAIGN-005 nombraba un dato que no existia en el modelo: campaigns.creator_budget_amount es nueva. Sobrecosto bloqueado, autorizable por finanzas con motivo obligatorio (ck_camp_budget_override).BR-CREATOR-008: el monto se fija al invitar y se congela al aceptar (tg_ccr_compromiso).DEC-103 a DEC-105.Corregido: el formulario de campana estaba copiado en cuatro clases de prueba (H-16, cuarta vez). Corregido: una foranea entre dos CHECK se quedaba huerfana de coma en la base sin-CHECK (1064).358 pruebas / 1201 aserciones. 1028 (MariaDB) y 1018 (MySQL 8) aserciones de restriccion.Las seis puertas en verde.
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -876,7 +876,7 @@
     <t xml:space="preserve">Seleccion, cupos por formato, costo comprometido por creador (congelado)</t>
   </si>
   <si>
-    <t xml:space="preserve">7.4 escribio la primera fila de campaign_creators y la protegio; falta el compromiso economico</t>
+    <t xml:space="preserve">docs/fase-7/7.5. DEC-103 a DEC-105. BR-CAMPAIGN-005 nombraba un dato que no existia. Cupos por mercado siguen siendo objetivo, no tope</t>
   </si>
   <si>
     <t xml:space="preserve">7.6</t>
@@ -885,7 +885,7 @@
     <t xml:space="preserve">Invitaciones: envio, expiracion, aceptacion, rechazo con motivo, preguntas</t>
   </si>
   <si>
-    <t xml:space="preserve">Tabla invitations lista. El envio depende de 4.9</t>
+    <t xml:space="preserve">BLOQUEADA por F4.9 (correo). El monto ya se fija y se congela (7.5); lo que falta es enviar</t>
   </si>
   <si>
     <t xml:space="preserve">7.7</t>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(Actividades!$H$2:$H$164,Actividades!$I$2:$I$164)/SUM(Actividades!$I$2:$I$164),0)</f>
-        <v>0.216049382716049</v>
+        <v>0.222222222222222</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">IFERROR(SUMPRODUCT($B$22:$B$25,$C$22:$C$25)/SUM($C$22:$C$25),0)</f>
-        <v>0.167426166208648</v>
+        <v>0.171391797404947</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2435,11 +2435,11 @@
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$G$2:$G$164,$A13)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">IFERROR($B13/COUNTA(Actividades!$A$2:$A$164),0)</f>
-        <v>0.165644171779141</v>
+        <v>0.171779141104294</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2461,11 +2461,11 @@
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$G$2:$G$164,$A15)</f>
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">IFERROR($B15/COUNTA(Actividades!$A$2:$A$164),0)</f>
-        <v>0.717791411042945</v>
+        <v>0.705521472392638</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$G$2:$G$164,$A16)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">IFERROR($B16/COUNTA(Actividades!$A$2:$A$164),0)</f>
-        <v>0.0122699386503067</v>
+        <v>0.0184049079754601</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2555,7 +2555,7 @@
       </c>
       <c r="B23" s="9" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Actividades!$B$2:$B$164=$A23)*Actividades!$H$2:$H$164*Actividades!$I$2:$I$164)/SUMPRODUCT((Actividades!$B$2:$B$164=$A23)*Actividades!$I$2:$I$164),0)</f>
-        <v>0.176470588235294</v>
+        <v>0.191176470588235</v>
       </c>
       <c r="C23" s="0" t="n">
         <v>12</v>
@@ -2566,7 +2566,7 @@
       </c>
       <c r="E23" s="8" t="n">
         <f aca="false">SUMPRODUCT((Actividades!$B$2:$B$164=$A23)*(Actividades!$G$2:$G$164="Terminado"))</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2780,7 +2780,7 @@
       </c>
       <c r="C36" s="9" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Actividades!$C$2:$C$164=$A36)*Actividades!$H$2:$H$164*Actividades!$I$2:$I$164)/SUMPRODUCT((Actividades!$C$2:$C$164=$A36)*Actividades!$I$2:$I$164),0)</f>
-        <v>0.392857142857143</v>
+        <v>0.464285714285714</v>
       </c>
       <c r="D36" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$C$2:$C$164,$A36)</f>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="E36" s="8" t="n">
         <f aca="false">SUMPRODUCT((Actividades!$C$2:$C$164=$A36)*(Actividades!$G$2:$G$164="Terminado"))</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5495,7 +5495,7 @@
         <v>280</v>
       </c>
     </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="21" t="n">
         <v>65</v>
       </c>
@@ -5515,11 +5515,11 @@
         <v>282</v>
       </c>
       <c r="G66" s="24" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H66" s="25" t="n">
         <f aca="false">IFERROR(INDEX(Config!$B$3:$B$8,MATCH($G66,Config!$A$3:$A$8,0)),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I66" s="26" t="n">
         <f aca="false">IFERROR(INDEX(Config!$C$3:$C$8,MATCH($G66,Config!$A$3:$A$8,0)),0)</f>
@@ -5549,7 +5549,7 @@
         <v>285</v>
       </c>
       <c r="G67" s="24" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H67" s="25" t="n">
         <f aca="false">IFERROR(INDEX(Config!$B$3:$B$8,MATCH($G67,Config!$A$3:$A$8,0)),0)</f>

</xml_diff>

<commit_message>
4.9: el correo (adelantado, desbloquea 7.6, 5.9, 4.1 y T-10)
Plantillas versionadas con vigencia: una publicada no se edita, se publica la siguiente y la anterior se cierra el dia antes (Periodo::sinSolape). email_log guarda plantilla, version, asunto y la HUELLA del cuerpo, no el cuerpo (DEC-106). Caida de idioma anotada, de ahi sale que falta traducir (DEC-107). Tres reintentos y failed visible con motivo, exigido por ck_el_failed (DEC-108). Corregido antes de produccion: Plantillas::vigente() resolvia por la columna puerta, que es 'la ultima publicada' y no 'la vigente' - una version programada dejaba un mes sin ninguna. Ahora se resuelve por periodo (T-21).Corregido: la opcion --version del comando chocaba con la de Symfony Console.380 pruebas / 1265 aserciones. 1070 (MariaDB) y 1060 (MySQL 8) aserciones de restriccion.Las seis puertas en verde.
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -621,7 +621,7 @@
     <t xml:space="preserve">Colas, scheduler, workers, Horizon</t>
   </si>
   <si>
-    <t xml:space="preserve">Las tablas jobs existen (esqueleto de Laravel); no hay ni un job propio</t>
+    <t xml:space="preserve">F4.9 estreno la cola: EnviarCorreo es el primer job propio, con QUEUE_CONNECTION=database. Faltan scheduler, supervisor y panel</t>
   </si>
   <si>
     <t xml:space="preserve">4.9</t>
@@ -630,7 +630,7 @@
     <t xml:space="preserve">Email: plantillas en BD con idioma/version/variables + Email Log + reintentos</t>
   </si>
   <si>
-    <t xml:space="preserve">Bloquea 4.1 (recuperacion), 5.9 (enlace de contrasena) y T-10</t>
+    <t xml:space="preserve">docs/fase-4/4.12-CORREO.md. DEC-106 a DEC-108. Adelantada porque bloqueaba 7.6, 5.9, 4.1 y T-10. Falta la cuenta de SMTP (Q-20)</t>
   </si>
   <si>
     <t xml:space="preserve">4.10</t>
@@ -885,7 +885,7 @@
     <t xml:space="preserve">Invitaciones: envio, expiracion, aceptacion, rechazo con motivo, preguntas</t>
   </si>
   <si>
-    <t xml:space="preserve">BLOQUEADA por F4.9 (correo). El monto ya se fija y se congela (7.5); lo que falta es enviar</t>
+    <t xml:space="preserve">Desbloqueada: F4.9 cerrada. El monto ya se fija y se congela (7.5)</t>
   </si>
   <si>
     <t xml:space="preserve">7.7</t>
@@ -2383,7 +2383,7 @@
       </c>
       <c r="B6" s="5" t="n">
         <f aca="false">IFERROR(SUMPRODUCT(Actividades!$H$2:$H$164,Actividades!$I$2:$I$164)/SUM(Actividades!$I$2:$I$164),0)</f>
-        <v>0.222222222222222</v>
+        <v>0.231481481481481</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2392,7 +2392,7 @@
       </c>
       <c r="B7" s="5" t="n">
         <f aca="false">IFERROR(SUMPRODUCT($B$22:$B$25,$C$22:$C$25)/SUM($C$22:$C$25),0)</f>
-        <v>0.171391797404947</v>
+        <v>0.178931714613699</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2435,11 +2435,11 @@
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$G$2:$G$164,$A13)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">IFERROR($B13/COUNTA(Actividades!$A$2:$A$164),0)</f>
-        <v>0.171779141104294</v>
+        <v>0.177914110429448</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2448,11 +2448,11 @@
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$G$2:$G$164,$A14)</f>
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">IFERROR($B14/COUNTA(Actividades!$A$2:$A$164),0)</f>
-        <v>0.098159509202454</v>
+        <v>0.104294478527607</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2461,11 +2461,11 @@
       </c>
       <c r="B15" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$G$2:$G$164,$A15)</f>
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">IFERROR($B15/COUNTA(Actividades!$A$2:$A$164),0)</f>
-        <v>0.705521472392638</v>
+        <v>0.699386503067485</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B16" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$G$2:$G$164,$A16)</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C16" s="9" t="n">
         <f aca="false">IFERROR($B16/COUNTA(Actividades!$A$2:$A$164),0)</f>
-        <v>0.0184049079754601</v>
+        <v>0.0122699386503067</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="B22" s="9" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Actividades!$B$2:$B$164=$A22)*Actividades!$H$2:$H$164*Actividades!$I$2:$I$164)/SUMPRODUCT((Actividades!$B$2:$B$164=$A22)*Actividades!$I$2:$I$164),0)</f>
-        <v>0.578947368421053</v>
+        <v>0.618421052631579</v>
       </c>
       <c r="C22" s="0" t="n">
         <v>8.5</v>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="E22" s="8" t="n">
         <f aca="false">SUMPRODUCT((Actividades!$B$2:$B$164=$A22)*(Actividades!$G$2:$G$164="Terminado"))</f>
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2720,7 +2720,7 @@
       </c>
       <c r="C33" s="9" t="n">
         <f aca="false">IFERROR(SUMPRODUCT((Actividades!$C$2:$C$164=$A33)*Actividades!$H$2:$H$164*Actividades!$I$2:$I$164)/SUMPRODUCT((Actividades!$C$2:$C$164=$A33)*Actividades!$I$2:$I$164),0)</f>
-        <v>0.40625</v>
+        <v>0.5</v>
       </c>
       <c r="D33" s="8" t="n">
         <f aca="false">COUNTIF(Actividades!$C$2:$C$164,$A33)</f>
@@ -2728,7 +2728,7 @@
       </c>
       <c r="E33" s="8" t="n">
         <f aca="false">SUMPRODUCT((Actividades!$C$2:$C$164=$A33)*(Actividades!$G$2:$G$164="Terminado"))</f>
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4453,7 +4453,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="21" t="n">
         <v>34</v>
       </c>
@@ -4473,11 +4473,11 @@
         <v>197</v>
       </c>
       <c r="G35" s="24" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H35" s="25" t="n">
         <f aca="false">IFERROR(INDEX(Config!$B$3:$B$8,MATCH($G35,Config!$A$3:$A$8,0)),0)</f>
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="I35" s="26" t="n">
         <f aca="false">IFERROR(INDEX(Config!$C$3:$C$8,MATCH($G35,Config!$A$3:$A$8,0)),0)</f>
@@ -4507,11 +4507,11 @@
         <v>200</v>
       </c>
       <c r="G36" s="24" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="H36" s="25" t="n">
         <f aca="false">IFERROR(INDEX(Config!$B$3:$B$8,MATCH($G36,Config!$A$3:$A$8,0)),0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I36" s="26" t="n">
         <f aca="false">IFERROR(INDEX(Config!$C$3:$C$8,MATCH($G36,Config!$A$3:$A$8,0)),0)</f>
@@ -5549,7 +5549,7 @@
         <v>285</v>
       </c>
       <c r="G67" s="24" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H67" s="25" t="n">
         <f aca="false">IFERROR(INDEX(Config!$B$3:$B$8,MATCH($G67,Config!$A$3:$A$8,0)),0)</f>

</xml_diff>

<commit_message>
7.6: invitaciones por enlace, plazo por campana y monto congelado
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -4992,7 +4992,7 @@
       </c>
       <c r="G67" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="H67" s="24">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="J67" s="22" t="inlineStr">
         <is>
-          <t>SIGUIENTE ITERACION PROPUESTA. Ya no tiene nada delante: 7.4 deja la lista corta, 7.5 el monto y F4.9 el correo. Decision pendiente: que pasa con el cupo cuando una invitacion caduca</t>
+          <t>docs/fase-7/7.6-INVITACIONES.md. DEC-119 a DEC-123. Enlace de un solo uso, plazo por campana, rechazo con motivo y reinvitacion con constancia. Las PREGUNTAS quedan fuera: T-38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
7.6b: enlace para usuarios internos (T-36), preguntas del creador (T-38) y dos 500 de pantalla
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -3009,7 +3009,7 @@
       </c>
       <c r="J25" s="22" t="inlineStr">
         <is>
-          <t>docs/fase-5/5.9-ENLACE-DE-CONTRASENA.md. DEC-113 a DEC-118. Recuperacion por enlace de 1 h, misma respuesta exista o no el correo, URL sin el token dentro. Falta la verificacion de correo</t>
+          <t>docs/fase-5/5.9 y docs/fase-7/7.6b. DEC-113 a DEC-118 y DEC-126. Recuperacion por enlace, misma respuesta exista o no el correo, URL sin token. Desde 7.6b tampoco se teclea la del equipo (BR-SEC-004 cerrada). Falta la verificacion de correo</t>
         </is>
       </c>
     </row>
@@ -5053,7 +5053,7 @@
       </c>
       <c r="J68" s="22" t="inlineStr">
         <is>
-          <t>La pantalla mas usada del sistema, segun el roadmap</t>
+          <t>SIGUIENTE ITERACION PROPUESTA. La pantalla mas usada del sistema, segun el roadmap. Ya no tiene nada delante</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
7.7: panel de seguimiento (embudo, cupos, dinero y alertas)
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -5040,7 +5040,7 @@
       </c>
       <c r="G68" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="H68" s="24">
@@ -5053,7 +5053,7 @@
       </c>
       <c r="J68" s="22" t="inlineStr">
         <is>
-          <t>SIGUIENTE ITERACION PROPUESTA. La pantalla mas usada del sistema, segun el roadmap. Ya no tiene nada delante</t>
+          <t>docs/fase-7/7.7-SEGUIMIENTO.md. DEC-127 y DEC-128. Embudo, cupo por mercado (cubierto = aceptado, no invitado), dinero con el margen detras de su permiso, y cuatro alertas</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
8.1: entregables, generados solos del brief del mercado
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -691,7 +691,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -755,7 +754,6 @@
         <v/>
       </c>
     </row>
-    <row r="10"/>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
@@ -870,7 +868,6 @@
         <v/>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
@@ -993,7 +990,6 @@
         <v/>
       </c>
     </row>
-    <row r="26"/>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
@@ -1460,7 +1456,6 @@
         <v/>
       </c>
     </row>
-    <row r="47"/>
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
@@ -5360,7 +5355,7 @@
       </c>
       <c r="G75" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="H75" s="24">
@@ -5373,7 +5368,7 @@
       </c>
       <c r="J75" s="22" t="inlineStr">
         <is>
-          <t>Tablas deliverables y deliverable_versions disenadas en 2.12</t>
+          <t>docs/fase-8/8.1-ENTREGABLES.md. DEC-129 a DEC-132. Se generan solos al aceptar, del brief EFECTIVO del mercado (N-03). Enlace https obligatorio + imagen opcional. Si faltan los hashtags del brief no se envia y se dice cuales. Portal del creador (/mis-entregas) con creator.portal, primer permiso de ambito EXTERNAL. 32 pruebas.</t>
         </is>
       </c>
     </row>
@@ -5408,7 +5403,7 @@
       </c>
       <c r="G76" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="H76" s="24">
@@ -5421,7 +5416,7 @@
       </c>
       <c r="J76" s="22" t="inlineStr">
         <is>
-          <t>Disenado en 2.12</t>
+          <t>docs/fase-8/8.2-VERSION-VIGENTE.md. DEC-137 y DEC-138. El append-only es de 8.1 (uq_dv_number con la fila bloqueada); 8.2 anade el puntero a la version APROBADA con clave ajena COMPUESTA --garantiza que la version es de ESE entregable-- y la reapertura con motivo de lista cerrada y firma, que no deshace nada. Ademas tg_dv_entregable_abierto: el veto de «no se entrega sobre algo cerrado» vivia en el servicio desde 8.1 y la base no lo conocia (T-47).</t>
         </is>
       </c>
     </row>
@@ -5456,7 +5451,7 @@
       </c>
       <c r="G77" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="H77" s="24">
@@ -5467,7 +5462,11 @@
         <f>IFERROR(INDEX(Config!$C$3:$C$8,MATCH($G77,Config!$A$3:$A$8,0)),0)</f>
         <v/>
       </c>
-      <c r="J77" s="22" t="inlineStr"/>
+      <c r="J77" s="22" t="inlineStr">
+        <is>
+          <t>docs/fase-8/8.3-REVISION.md. DEC-133 a DEC-136. Bandeja GLOBAL ordenada por lo que lleva mas esperando. Solo las rondas del CLIENTE cuentan y son POR ENTREGABLE (el contador estaba en campaign_creators). Pasarse bloquea y exige decidir si se cobra o se absorbe, firmado. Tres permisos: content.review, content.approve y content.extra_round. tg_cvw_inmutable cierra el append-only que 2.12 afirmaba sin impedir nada. 30 pruebas.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="20" t="n">
@@ -5500,7 +5499,7 @@
       </c>
       <c r="G78" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>En curso</t>
         </is>
       </c>
       <c r="H78" s="24">
@@ -5513,7 +5512,7 @@
       </c>
       <c r="J78" s="22" t="inlineStr">
         <is>
-          <t>included_revision_rounds ya se guarda en la campana</t>
+          <t>included_revision_rounds se cuenta y se impone desde 8.3, por entregable y solo con las rondas del cliente. Queda el limite duro: hoy se puede pasar tantas veces como haga falta mientras se decida y se firme cada una.</t>
         </is>
       </c>
     </row>
@@ -5592,7 +5591,7 @@
       </c>
       <c r="G80" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="H80" s="24">
@@ -5603,7 +5602,11 @@
         <f>IFERROR(INDEX(Config!$C$3:$C$8,MATCH($G80,Config!$A$3:$A$8,0)),0)</f>
         <v/>
       </c>
-      <c r="J80" s="22" t="inlineStr"/>
+      <c r="J80" s="22" t="inlineStr">
+        <is>
+          <t>docs/fase-8/8.6-PUBLICACION.md. DEC-139 a DEC-141. El creador pega el enlace desde su portal y el equipo puede hacerlo por el; solo se publica lo APROBADO y esa version (snapshot con clave ajena compuesta). La red se deduce del enlace con platforms.url_pattern y tiene que ser la del brief. La huella normaliza la URL para que uq_pub_fingerprint sirva de algo. 31 pruebas. La PROGRAMACION queda fuera: hoy se registra lo ya publicado.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="20" t="n">

</xml_diff>

<commit_message>
8.1-8.7: entregables, revision, version vigente, publicacion y evidencia
8.1 entregables y versiones - 8.3 revision con rondas y firma - 8.2 puntero a version aprobada con FK compuesta - 8.6 registro de publicacion - 8.7 evidencia y verificacion (viva_gate). Protocolo de entrega y disparador de CI para ramas feat/**. 659 tests, 1.438 aserciones SQL, seis puertas verdes.
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -5639,7 +5639,7 @@
       </c>
       <c r="G81" s="23" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Terminado</t>
         </is>
       </c>
       <c r="H81" s="24">
@@ -5652,7 +5652,7 @@
       </c>
       <c r="J81" s="22" t="inlineStr">
         <is>
-          <t>Tabla publication_evidence disenada</t>
+          <t>docs/fase-8/8.7-EVIDENCIA.md. DEC-142 a DEC-144. La evidencia es una CAPTURA y no una comprobacion HTTP: Instagram y TikTok responden igual a un post vivo que a un bloqueo, y de verified cuelga el pago. Permiso propio content.verify. Si el post no esta, el entregable vuelve al CREADOR y se le avisa. permanence_until se calcula al verificar. T-50: una rechazada bloqueaba su propio enlace (columna puerta viva_gate, la decimoquinta). 21 pruebas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T-77: el sembrador no reescribe lo configurado ni se para con un periodo cerrado
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -10552,7 +10552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="35" min="1" max="1"/>
@@ -12853,6 +12853,39 @@
       <c r="G70" s="69" t="inlineStr">
         <is>
           <t>verificar-migraciones.py acuso a document_series de crear la columna document_type de mas: la migracion de 9.12 suelta la tabla y la vuelve a crear con otra forma, pero el doble de Schema no soltaba nada, asi que el grabador recogia la union de las dos formas. Mismo archivo, mismo motivo y misma familia que T-75. La leccion: cada doble vacio del grabador es un falso positivo esperando, y un verificador que da rojo por algo que esta bien acaba ignorado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="67" t="inlineStr">
+        <is>
+          <t>T-77</t>
+        </is>
+      </c>
+      <c r="B71" s="68" t="inlineStr">
+        <is>
+          <t>Resuelta</t>
+        </is>
+      </c>
+      <c r="C71" s="68" t="n"/>
+      <c r="D71" s="69" t="inlineStr">
+        <is>
+          <t>RESUELTA (2026-08-31, hotfix de 9.12). El sembrador reescribia lo que una persona ya habia configurado, y ademas reventaba.</t>
+        </is>
+      </c>
+      <c r="E71" s="69" t="inlineStr">
+        <is>
+          <t>9.12 (hotfix)</t>
+        </is>
+      </c>
+      <c r="F71" s="69" t="inlineStr">
+        <is>
+          <t>Equipo de desarrollo</t>
+        </is>
+      </c>
+      <c r="G71" s="69" t="inlineStr">
+        <is>
+          <t>Reportada desde la instalacion: db:seed se paro con un 45000 porque updateOrInsert movia el valid_from de la fila ABIERTA de fx_official_sources encima de un periodo cerrado a mano (T-73 desde el otro lado). Lo que el error tapaba era peor: el sembrador murio en la linea 71 de 700, asi que los proveedores de 9.17d y los tipos de comprobante de 9.12 no llegaron a entrar. Y de fondo: cada db:seed --lo que el runbook manda tras cada migracion-- devolvia a fabrica el nombre, lema, colores y tipografia de la marca y la direccion de la sociedad, REGENERABA sus uuid y reactivaba fuentes y proveedores apagados a proposito. Regla nueva: lo que una persona puede cambiar se siembra si falta y no se toca si esta (sembrarSiFalta); donde hay vigencia, el periodo empieza el dia siguiente al ultimo cierre. 5 pruebas verificadas en rojo sin el arreglo.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
T-81: dos URLs escritas a mano en bootstrap/app.php rompian el acceso desde 9.21a
</commit_message>
<xml_diff>
--- a/docs/LATAM-Social-avance.xlsx
+++ b/docs/LATAM-Social-avance.xlsx
@@ -10852,7 +10852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:G75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="8" customWidth="1" style="35" min="1" max="1"/>
@@ -13293,6 +13293,39 @@
       <c r="G74" s="69" t="inlineStr">
         <is>
           <t>Reportado desde la instalacion: «el entrar me lleva a NOT FOUND». La sesion abria bien; fallaba el destino. redirect()-&gt;intended() obedece a la direccion guardada en la sesion aunque ya no exista, y desde 9.21a hay 149 que no existen: toda sesion abierta antes de desplegar la mudanza a /backoffice lleva guardado un /panel o un /creadores que hoy son 404. Le pasa a TODO EL MUNDO el dia del despliegue y a cada uno una sola vez, que es la peor forma de un fallo: se arregla solo antes de que nadie lo pueda reproducir. Ahora la direccion guardada tiene que ser del propio dominio y seguir resolviendo --se le pregunta al enrutador--; si no, al panel. Tambien se rechaza la que existe con otro verbo. 5 pruebas, 3 verificadas en rojo sin el arreglo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="67" t="inlineStr">
+        <is>
+          <t>T-81</t>
+        </is>
+      </c>
+      <c r="B75" s="68" t="inlineStr">
+        <is>
+          <t>Resuelta</t>
+        </is>
+      </c>
+      <c r="C75" s="68" t="n"/>
+      <c r="D75" s="69" t="inlineStr">
+        <is>
+          <t>RESUELTA (2026-09-01, hotfix de 9.9b). La causa de verdad del 404 al entrar: dos URLs escritas a mano en bootstrap/app.php.</t>
+        </is>
+      </c>
+      <c r="E75" s="69" t="inlineStr">
+        <is>
+          <t>9.9b (hotfix)</t>
+        </is>
+      </c>
+      <c r="F75" s="69" t="inlineStr">
+        <is>
+          <t>Equipo de desarrollo</t>
+        </is>
+      </c>
+      <c r="G75" s="69" t="inlineStr">
+        <is>
+          <t>T-80 arreglo una mitad (el url.intended viejo) y el fallo siguio. La otra era redirectUsersTo(/panel): quien YA tenia sesion y pulsaba Entrar caia en el middleware guest, que lo mandaba a /panel, que desde la mudanza no existe. 9.21a presumio de «ni una URL que corregir» y era casi verdad: docs/08 prohibe escribir URLs en las VISTAS, asi que las 149 pantallas se mudaron solas; nadie miro bootstrap/, que no es una vista, y la busqueda de entonces solo cubrio app/, resources/ y config/. Debajo habia algo peor: sincronizar NUNCA copiaba stage/bootstrap/, asi que ese directorio del arbol de entrega llevaba desde el 25 de agosto sin actualizarse --providers.php sin Campaign, Content ni Finance-- y nada de lo que hay dentro se probaba jamas. Ahora las dos direcciones salen del enrutador, sincronizar copia bootstrap/, y una prueba recorre bootstrap/ y config/ exigiendo que toda direccion escrita a mano la reconozca el enrutador. 8 pruebas, 2 verificadas en rojo sin el arreglo.</t>
         </is>
       </c>
     </row>

</xml_diff>